<commit_message>
feat: refine evaluation engine (load balancing, timezone window) and update evaluators data
</commit_message>
<xml_diff>
--- a/Evaluators.xlsx
+++ b/Evaluators.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sap-my.sharepoint.com/personal/carlos_edgar_moreno_sap_com/Documents/CEM/2026/03 Mar/02 Projects/020 Scheduling App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="8_{707C9252-19BB-E042-9FC5-4144E6F268D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{733B3BEA-3B29-3244-BEDA-D0F0E7C24C2B}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="8_{707C9252-19BB-E042-9FC5-4144E6F268D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81D715E5-47C7-3545-BCB8-DC4B4B93EE22}"/>
   <bookViews>
-    <workbookView xWindow="8980" yWindow="-19720" windowWidth="27640" windowHeight="16680" xr2:uid="{FF3BE242-5C07-A14B-B847-4B4B85AB18A9}"/>
+    <workbookView xWindow="5120" yWindow="660" windowWidth="13800" windowHeight="18980" xr2:uid="{FF3BE242-5C07-A14B-B847-4B4B85AB18A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="58">
   <si>
     <t>Faculty Name</t>
   </si>
@@ -74,15 +74,6 @@
     <t>Germany</t>
   </si>
   <si>
-    <t>Amy Hawkins</t>
-  </si>
-  <si>
-    <t>Perth</t>
-  </si>
-  <si>
-    <t>Australia</t>
-  </si>
-  <si>
     <t>Nelly Rebollo</t>
   </si>
   <si>
@@ -207,6 +198,18 @@
   </si>
   <si>
     <t>Berlin</t>
+  </si>
+  <si>
+    <t>Hedda Samia</t>
+  </si>
+  <si>
+    <t>Aarohi Tamhane</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>India</t>
   </si>
 </sst>
 </file>
@@ -267,6 +270,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -586,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD3BC18-E400-F847-B70F-FFFFE5A1DC73}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.33203125" customWidth="1"/>
@@ -605,7 +612,7 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -619,7 +626,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -633,7 +640,7 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -647,54 +654,54 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
@@ -703,12 +710,12 @@
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
@@ -717,236 +724,236 @@
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="s">
         <v>5</v>
       </c>
-      <c r="D16" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" t="s">
-        <v>33</v>
-      </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D19" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D23" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="C25" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D25" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B26" t="s">
         <v>10</v>
@@ -955,21 +962,35 @@
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="C27" t="s">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>41</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>